<commit_message>
Update investigaciones, i115 espacios actividad fisica
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -2785,7 +2785,11 @@
           <t>Índice de condiciones de reconciliación en Bogotá D.C.</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>El Índice de Condiciones de Reconciliación en Bogotá D.C., es una herramienta que mide cómo avanza la reconciliación en la ciudad. A partir de dimensiones como cohesión social, inclusión, memoria y cultura política, analiza percepciones y actitudes ciudadanas frente a la convivencia y la paz. Sus resultados orientan decisiones públicas y fortalecen la construcción de confianza y tejido social en Bogotá.</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>Sector</t>
@@ -21041,7 +21045,7 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1uvPcjC3VFFwdTN4LKTZqQa4dd_mt6aRq/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1Zr6q_Eutt4lnN9Y6OUXIpAcfFvHJKFJ2/view?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -22174,10 +22178,26 @@
       <c r="A651" t="n">
         <v>115</v>
       </c>
-      <c r="B651" t="inlineStr"/>
-      <c r="C651" t="inlineStr"/>
-      <c r="D651" t="inlineStr"/>
-      <c r="E651" t="inlineStr"/>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Informe final</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informe final </t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1BVdsnc2YA1a2JeXAjjW5O6Z2t0UkP55Z-0WtShl4xa8/edit?usp=sharing</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" t="n">

</xml_diff>

<commit_message>
Update investigaciones, i104, i106, i119
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -20685,12 +20685,12 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>Informe Festival Monumentum 2025</t>
+          <t>Productos finales Festival Monumentum 2025</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
@@ -20700,7 +20700,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UVUUqWPRqoC9-J_3rJPCiwC_FLLGKNPY/view?usp=sharing</t>
+          <t>https://drive.google.com/drive/folders/16LFLVNlKGuWbgTUXHDjiWESjGmAAQM1L?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -20708,51 +20708,19 @@
       <c r="A581" t="n">
         <v>104</v>
       </c>
-      <c r="B581" t="inlineStr">
-        <is>
-          <t>Presentación</t>
-        </is>
-      </c>
-      <c r="C581" t="inlineStr">
-        <is>
-          <t>Presentación resultados Festival Monumentum 2025</t>
-        </is>
-      </c>
-      <c r="D581" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E581" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1Xe170cnqUJe0L75fIRULax6fAtG4DoW9/view?usp=sharing</t>
-        </is>
-      </c>
+      <c r="B581" t="inlineStr"/>
+      <c r="C581" t="inlineStr"/>
+      <c r="D581" t="inlineStr"/>
+      <c r="E581" t="inlineStr"/>
     </row>
     <row r="582">
       <c r="A582" t="n">
         <v>104</v>
       </c>
-      <c r="B582" t="inlineStr">
-        <is>
-          <t>Instrumento recolección</t>
-        </is>
-      </c>
-      <c r="C582" t="inlineStr">
-        <is>
-          <t>Formularios Festival Monumentum 2025</t>
-        </is>
-      </c>
-      <c r="D582" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E582" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1gnrVe2NjozYAHQCAlLTR23iZjIlgxno0/view?usp=sharing</t>
-        </is>
-      </c>
+      <c r="B582" t="inlineStr"/>
+      <c r="C582" t="inlineStr"/>
+      <c r="D582" t="inlineStr"/>
+      <c r="E582" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" t="n">
@@ -20937,12 +20905,12 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>Informe Premio Luis Caballero 2025</t>
+          <t>Productos finales Premio Luis Caballero 2025</t>
         </is>
       </c>
       <c r="D592" t="inlineStr">
@@ -20952,7 +20920,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/18QKMBaJoy4nqZQlFRNYvsZzoo_sFJDIT/view?usp=sharing</t>
+          <t>https://drive.google.com/drive/folders/15KsNtJH-r9FD1xvh9vzNj-9Df_ikXVnD?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -20960,51 +20928,19 @@
       <c r="A593" t="n">
         <v>106</v>
       </c>
-      <c r="B593" t="inlineStr">
-        <is>
-          <t>Presentación</t>
-        </is>
-      </c>
-      <c r="C593" t="inlineStr">
-        <is>
-          <t>Presentación resultados Premio Luis Caballero 2025</t>
-        </is>
-      </c>
-      <c r="D593" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E593" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hqNl-FukfRsmkLFkKFbhRMjbCi_keQVa/view?usp=sharing</t>
-        </is>
-      </c>
+      <c r="B593" t="inlineStr"/>
+      <c r="C593" t="inlineStr"/>
+      <c r="D593" t="inlineStr"/>
+      <c r="E593" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" t="n">
         <v>106</v>
       </c>
-      <c r="B594" t="inlineStr">
-        <is>
-          <t>Instrumento recolección</t>
-        </is>
-      </c>
-      <c r="C594" t="inlineStr">
-        <is>
-          <t>Formularios Premio Luis Caballero 2025</t>
-        </is>
-      </c>
-      <c r="D594" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E594" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1yzZXgr7VzlUbRtj5fNNi_JyDWjan8aNY/view?usp=sharing</t>
-        </is>
-      </c>
+      <c r="B594" t="inlineStr"/>
+      <c r="C594" t="inlineStr"/>
+      <c r="D594" t="inlineStr"/>
+      <c r="E594" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" t="n">
@@ -22205,12 +22141,12 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Carpeta archivos</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Bases de datos depuras Ciclovía y Escuela de la Bici</t>
+          <t>Informe presentación resultados programas de Ciclovía y Escuela de la bici</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -22220,7 +22156,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1E04LKSNgVLJxshdGwwWy8BQRzbJwMkGs/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1ml0N-5tIACWRSjSXde5tKA2Q9Wn_J-9k/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22230,12 +22166,12 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>Informe presentación resultados programas de Ciclovía y Escuela de la bici</t>
+          <t>Instrumento de recolección Ciclovía 2025</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
@@ -22245,7 +22181,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ml0N-5tIACWRSjSXde5tKA2Q9Wn_J-9k/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1uwG-2pHQMS6-t0GhwSTGLJ3fWap6L6Y6/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22255,12 +22191,12 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Tabla de resultado Escuela de la Bici</t>
+          <t>Instrumento de recolección Escuela de la Bici</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
@@ -22270,7 +22206,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1zQZjjzdyGr9BkltBh0Xu5ntzvtJ1siUK/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1j44f0nt3hcD7HjD-Ya48stCgjyv2gPDm/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22305,12 +22241,12 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Escuela de la Bici</t>
+          <t>Tabla de resultado Escuela de la Bici</t>
         </is>
       </c>
       <c r="D656" t="inlineStr">
@@ -22320,7 +22256,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1j44f0nt3hcD7HjD-Ya48stCgjyv2gPDm/view?usp=drive_link</t>
+          <t>https://docs.google.com/spreadsheets/d/1zQZjjzdyGr9BkltBh0Xu5ntzvtJ1siUK/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
@@ -22330,12 +22266,12 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Ciclovía 2025</t>
+          <t>Bases de datos depuras Ciclovía y Escuela de la Bici</t>
         </is>
       </c>
       <c r="D657" t="inlineStr">
@@ -22345,7 +22281,7 @@
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1uwG-2pHQMS6-t0GhwSTGLJ3fWap6L6Y6/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1E04LKSNgVLJxshdGwwWy8BQRzbJwMkGs/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22584,12 +22520,12 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>Informe Festival de Verano 2025</t>
+          <t>Productos finales Festival de Verano 2025</t>
         </is>
       </c>
       <c r="D670" t="inlineStr">
@@ -22599,7 +22535,7 @@
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1flNJJ6CFGtqXgQG3sAJJHbyuCFh8RuOs/view?usp=sharing</t>
+          <t>https://drive.google.com/drive/folders/14Ap2CtsPvGqgr55CTIh_z0MO3XnfklKi?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -22607,26 +22543,10 @@
       <c r="A671" t="n">
         <v>119</v>
       </c>
-      <c r="B671" t="inlineStr">
-        <is>
-          <t>Instrumento recolección</t>
-        </is>
-      </c>
-      <c r="C671" t="inlineStr">
-        <is>
-          <t>Formularios Festival de Verano 2025</t>
-        </is>
-      </c>
-      <c r="D671" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E671" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1syhJzh5ipnYrYWpHmXhOuq1UKOuyL5FQ/view?usp=sharing</t>
-        </is>
-      </c>
+      <c r="B671" t="inlineStr"/>
+      <c r="C671" t="inlineStr"/>
+      <c r="D671" t="inlineStr"/>
+      <c r="E671" t="inlineStr"/>
     </row>
     <row r="672">
       <c r="A672" t="n">
@@ -22772,12 +22692,12 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>Instrucciones sobre registro de información</t>
+          <t>Tablero Encuesta</t>
         </is>
       </c>
       <c r="D682" t="inlineStr">
@@ -22787,7 +22707,7 @@
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1gbIyrWH8cK07q00yoPBs9D8IWYNv4P2I/view?usp=drive_link</t>
+          <t>https://lookerstudio.google.com/reporting/ccbecff5-f250-4a21-b1f8-5290632c1187/page/p_shhgwuepsd</t>
         </is>
       </c>
     </row>
@@ -22797,12 +22717,12 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>Prototipo para registro</t>
+          <t>Instrucciones sobre registro de información</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
@@ -22812,7 +22732,7 @@
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>https://www.prototipos-sicc.com/app/barrios_vivos/explorar</t>
+          <t>https://drive.google.com/file/d/1gbIyrWH8cK07q00yoPBs9D8IWYNv4P2I/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22822,12 +22742,12 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>Tablero de seguimiento</t>
+          <t>Prototipo para registro</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -22837,7 +22757,7 @@
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>https://lookerstudio.google.com/reporting/a1e266a6-ed1a-4500-8776-58e82d1d7746/page/p_pjg06p6njd</t>
+          <t>https://www.prototipos-sicc.com/app/barrios_vivos/explorar</t>
         </is>
       </c>
     </row>
@@ -22847,12 +22767,12 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Audiovisual</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>Vídeo tutoriales para registro</t>
+          <t>Tablero de seguimiento</t>
         </is>
       </c>
       <c r="D685" t="inlineStr">
@@ -22862,7 +22782,7 @@
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1Cuy0w3cr883zTx_4X1n4TquCUCnheBRm</t>
+          <t>https://lookerstudio.google.com/reporting/a1e266a6-ed1a-4500-8776-58e82d1d7746/page/p_pjg06p6njd</t>
         </is>
       </c>
     </row>
@@ -22872,12 +22792,12 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Audiovisual</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>Tablero Encuesta</t>
+          <t>Vídeo tutoriales para registro</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
@@ -22887,7 +22807,7 @@
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>https://lookerstudio.google.com/reporting/ccbecff5-f250-4a21-b1f8-5290632c1187/page/p_shhgwuepsd</t>
+          <t>https://drive.google.com/drive/folders/1Cuy0w3cr883zTx_4X1n4TquCUCnheBRm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update investigaciones, i113 productos y descripcion
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EBC - LEO 2025</t>
+          <t>EBC - Encuesta de Lectura, Escritura y Oralidad 2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Lectura - Escritura - Oralidad -EBC</t>
+          <t>lectura, bibliotecas, oralidad, podcast, libros, escritura, espacios de lectura, virgilio barco, bibliored</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -8615,7 +8615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E730"/>
+  <dimension ref="A1:E732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21732,16 +21732,16 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Espacios de Lectura</t>
+          <t>Tabero de Resultados</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
@@ -21751,22 +21751,22 @@
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16W6G5tRSMAk7F6SDasy_0yM92zpbwTbq/view?usp=drive_link</t>
+          <t>https://observatoriocultura.github.io/observatorio/#/ebc/lectura-escritura-y-oralidad-2025</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Usaquén - Servitá</t>
+          <t>Base de datos detallada</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
@@ -21776,7 +21776,7 @@
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FRWQBJGGoZZttLVMLwagnXXYShR2lFqi/view?usp=drive_link</t>
+          <t>https://docs.google.com/spreadsheets/d/1ncjBs9trvq52fX5STxFHJTkdM7tQLgc6/edit?usp=drive_link&amp;ouid=114299960211627169695&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
@@ -21786,12 +21786,12 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública La Peña</t>
+          <t>Instrumento de recolección Espacios de Lectura</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
@@ -21801,7 +21801,7 @@
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1RwsGRlcn7XYuXJ1rtmYJUnWj69aEpyMV/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/16W6G5tRSMAk7F6SDasy_0yM92zpbwTbq/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21816,7 +21816,7 @@
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública FUGA</t>
+          <t>Sondeo Visitantes Biblioteca Pública Usaquén - Servitá</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
@@ -21826,7 +21826,7 @@
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DYP4zsQhzkx8PH-yydqgAloHd_DCEsTV/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1FRWQBJGGoZZttLVMLwagnXXYShR2lFqi/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21841,7 +21841,7 @@
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Virgilio Barco</t>
+          <t>Sondeo Visitantes Biblioteca Pública La Peña</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
@@ -21851,7 +21851,7 @@
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1caNM182qy71k48IqO5Mzv168P1KIbDs-/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1RwsGRlcn7XYuXJ1rtmYJUnWj69aEpyMV/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21866,7 +21866,7 @@
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Caros E. Restrepo</t>
+          <t>Sondeo Visitantes Biblioteca Pública FUGA</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19dgvioy6RYxY0oUSvS7HrWGkCn6Bdcve/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1DYP4zsQhzkx8PH-yydqgAloHd_DCEsTV/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21891,7 +21891,7 @@
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Francisco José de Caldas</t>
+          <t>Sondeo Visitantes Biblioteca Pública Virgilio Barco</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
@@ -21901,7 +21901,7 @@
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Xdo-9N2TnWtBpoKVhiMIb3Cwj2SYmDWR/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1caNM182qy71k48IqO5Mzv168P1KIbDs-/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21916,7 +21916,7 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Gabriel García Márquez - El Tunal</t>
+          <t>Sondeo Visitantes Biblioteca Pública Caros E. Restrepo</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
@@ -21926,7 +21926,7 @@
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-_wpdpR7e4SMEdEdCVZQNFsVSxxFf7Yn/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/19dgvioy6RYxY0oUSvS7HrWGkCn6Bdcve/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21941,7 +21941,7 @@
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Julio Mario Santodomingo</t>
+          <t>Sondeo Visitantes Biblioteca Pública Francisco José de Caldas</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
@@ -21951,7 +21951,7 @@
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19-EGROjB7Se6H5BC7lQ-5kcioDv17Aj8/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1Xdo-9N2TnWtBpoKVhiMIb3Cwj2SYmDWR/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21966,7 +21966,7 @@
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>Sondeo Visitantes Biblioteca Pública Manuel Zapata Olivella - El Tintal</t>
+          <t>Sondeo Visitantes Biblioteca Pública Gabriel García Márquez - El Tunal</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
@@ -21976,7 +21976,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1smpXVkZNK0D0NVvXTpaToUpQYbnUsJ2X/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1-_wpdpR7e4SMEdEdCVZQNFsVSxxFf7Yn/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -21984,14 +21984,30 @@
       <c r="A645" t="n">
         <v>114</v>
       </c>
-      <c r="B645" t="inlineStr"/>
-      <c r="C645" t="inlineStr"/>
-      <c r="D645" t="inlineStr"/>
-      <c r="E645" t="inlineStr"/>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Informe final</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Sondeo Visitantes Biblioteca Pública Julio Mario Santodomingo</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/19-EGROjB7Se6H5BC7lQ-5kcioDv17Aj8/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
@@ -22000,7 +22016,7 @@
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>Informe Espacios de actividad física</t>
+          <t>Sondeo Visitantes Biblioteca Pública Manuel Zapata Olivella - El Tintal</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
@@ -22008,57 +22024,33 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E646" t="inlineStr"/>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1smpXVkZNK0D0NVvXTpaToUpQYbnUsJ2X/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>115</v>
-      </c>
-      <c r="B647" t="inlineStr">
-        <is>
-          <t>Presentación</t>
-        </is>
-      </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>Presentación resultados programas de Espacios de actividad física</t>
-        </is>
-      </c>
-      <c r="D647" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E647" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1qlsGIDoE8xuZRs0DD2wbob15tro_VEMX/view?usp=drive_link</t>
-        </is>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="B647" t="inlineStr"/>
+      <c r="C647" t="inlineStr"/>
+      <c r="D647" t="inlineStr"/>
+      <c r="E647" t="inlineStr"/>
     </row>
     <row r="648">
       <c r="A648" t="n">
         <v>115</v>
       </c>
-      <c r="B648" t="inlineStr">
-        <is>
-          <t>Informe cuantitativo</t>
-        </is>
-      </c>
-      <c r="C648" t="inlineStr">
-        <is>
-          <t>Tablas de resultado Espacios de actividad física</t>
-        </is>
-      </c>
+      <c r="B648" t="inlineStr"/>
+      <c r="C648" t="inlineStr"/>
       <c r="D648" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="E648" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1PeAnosF7Ne2O-rSJHyJNPYU_8VyKObOM/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
-        </is>
-      </c>
+      <c r="E648" t="inlineStr"/>
     </row>
     <row r="649">
       <c r="A649" t="n">
@@ -22066,22 +22058,22 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>Base de datos Espacios de actividad física</t>
+          <t>Presentación resultados programas de Espacios de actividad física</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1pkjosapWgOR6hhHYZF-HqbqKBJZlYhtM/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1qlsGIDoE8xuZRs0DD2wbob15tro_VEMX/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22091,12 +22083,12 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Espacios de actividad física</t>
+          <t>Tablas de resultado Espacios de actividad física</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
@@ -22106,7 +22098,7 @@
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1u4nc5ifpincy8njQifsXd-QfzDxYlwR8/view?usp=drive_link</t>
+          <t>https://docs.google.com/spreadsheets/d/1PeAnosF7Ne2O-rSJHyJNPYU_8VyKObOM/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
@@ -22116,12 +22108,12 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t xml:space="preserve">Informe final </t>
+          <t>Base de datos Espacios de actividad física</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
@@ -22131,22 +22123,22 @@
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>https://docs.google.com/document/d/1BVdsnc2YA1a2JeXAjjW5O6Z2t0UkP55Z-0WtShl4xa8/edit?usp=sharing</t>
+          <t>https://docs.google.com/spreadsheets/d/1pkjosapWgOR6hhHYZF-HqbqKBJZlYhtM/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Informe presentación resultados programas de Ciclovía y Escuela de la bici</t>
+          <t>Instrumento de recolección Espacios de actividad física</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -22156,22 +22148,22 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ml0N-5tIACWRSjSXde5tKA2Q9Wn_J-9k/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1u4nc5ifpincy8njQifsXd-QfzDxYlwR8/view?usp=drive_link</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Ciclovía 2025</t>
+          <t>Informe final Espacios de actividad física</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
@@ -22181,7 +22173,7 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1uwG-2pHQMS6-t0GhwSTGLJ3fWap6L6Y6/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1VMhbyOIs4ScBC_JIaaLKz8_A-A7G5cOl/view?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -22191,12 +22183,12 @@
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Instrumento de recolección Escuela de la Bici</t>
+          <t>Informe presentación resultados programas de Ciclovía y Escuela de la bici</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
@@ -22206,7 +22198,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1j44f0nt3hcD7HjD-Ya48stCgjyv2gPDm/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1ml0N-5tIACWRSjSXde5tKA2Q9Wn_J-9k/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22216,12 +22208,12 @@
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>Tabla de resultado Ciclovía 2025</t>
+          <t>Instrumento de recolección Ciclovía 2025</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
@@ -22231,7 +22223,7 @@
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/16ZpRSW0DGRb8JPE9QCzrLu2VyFN2IXTt/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1uwG-2pHQMS6-t0GhwSTGLJ3fWap6L6Y6/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22241,12 +22233,12 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
         <is>
-          <t>Tabla de resultado Escuela de la Bici</t>
+          <t>Instrumento de recolección Escuela de la Bici</t>
         </is>
       </c>
       <c r="D656" t="inlineStr">
@@ -22256,7 +22248,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1zQZjjzdyGr9BkltBh0Xu5ntzvtJ1siUK/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1j44f0nt3hcD7HjD-Ya48stCgjyv2gPDm/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22266,12 +22258,12 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Carpeta archivos</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>Bases de datos depuras Ciclovía y Escuela de la Bici</t>
+          <t>Tabla de resultado Ciclovía 2025</t>
         </is>
       </c>
       <c r="D657" t="inlineStr">
@@ -22281,22 +22273,22 @@
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1E04LKSNgVLJxshdGwwWy8BQRzbJwMkGs/view?usp=drive_link</t>
+          <t>https://docs.google.com/spreadsheets/d/16ZpRSW0DGRb8JPE9QCzrLu2VyFN2IXTt/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>Docuento metodológico</t>
+          <t>Tabla de resultado Escuela de la Bici</t>
         </is>
       </c>
       <c r="D658" t="inlineStr">
@@ -22306,22 +22298,22 @@
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aRQvwNu04n8HAXbE9o69GhoBogD2Uqj6/view?usp=sharing</t>
+          <t>https://docs.google.com/spreadsheets/d/1zQZjjzdyGr9BkltBh0Xu5ntzvtJ1siUK/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>Instrumento de recolección</t>
+          <t>Bases de datos depuras Ciclovía y Escuela de la Bici</t>
         </is>
       </c>
       <c r="D659" t="inlineStr">
@@ -22331,7 +22323,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1VZIqZvzrUOBhPEVGF_n98ZthOb8RmV4V/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1E04LKSNgVLJxshdGwwWy8BQRzbJwMkGs/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22341,12 +22333,12 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>Anexo</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>Matriz de revisión de literatura</t>
+          <t>Docuento metodológico</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
@@ -22356,7 +22348,7 @@
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1U5vso-3VmBTA0uPp6Jwz3zolvbWR17sT/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1aRQvwNu04n8HAXbE9o69GhoBogD2Uqj6/view?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -22366,13 +22358,12 @@
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>Anexo</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t xml:space="preserve">Matriz de tipología de actores
-</t>
+          <t>Instrumento de recolección</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
@@ -22382,7 +22373,7 @@
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HQUAEOPZWxBtWc-dexksGmXsqH3VLyB3/view?usp=drive_link</t>
+          <t>https://docs.google.com/spreadsheets/d/1VZIqZvzrUOBhPEVGF_n98ZthOb8RmV4V/edit?usp=drive_link&amp;ouid=114639277514087565011&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
@@ -22397,7 +22388,7 @@
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>Matriz de esquema interpretativo de la gobernanza del deporte</t>
+          <t>Matriz de revisión de literatura</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
@@ -22407,7 +22398,7 @@
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16EFX41hHQvz_pSfEG86A1RV2KQ969hzt/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1U5vso-3VmBTA0uPp6Jwz3zolvbWR17sT/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22417,37 +22408,38 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>Plan de trabajo</t>
+          <t>Anexo</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
         <is>
-          <t>Plan de trabajo</t>
+          <t xml:space="preserve">Matriz de tipología de actores
+</t>
         </is>
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1t70D31QSK9xXUEgVSMhUzuwxOwgYAfyO/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1HQUAEOPZWxBtWc-dexksGmXsqH3VLyB3/view?usp=drive_link</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Anexo</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>Formulario EBC - PACCP Final</t>
+          <t>Matriz de esquema interpretativo de la gobernanza del deporte</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
@@ -22457,22 +22449,34 @@
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1qsclq1ogNVWTc6Sh7swGgV-k7DZr-Wnj/edit?usp=drive_link&amp;ouid=105090632649587320414&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/16EFX41hHQvz_pSfEG86A1RV2KQ969hzt/view?usp=drive_link</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>Base de datos</t>
-        </is>
-      </c>
-      <c r="C665" t="inlineStr"/>
-      <c r="D665" t="inlineStr"/>
-      <c r="E665" t="inlineStr"/>
+          <t>Plan de trabajo</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Plan de trabajo</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1t70D31QSK9xXUEgVSMhUzuwxOwgYAfyO/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="666">
       <c r="A666" t="n">
@@ -22480,18 +22484,34 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
-        </is>
-      </c>
-      <c r="C666" t="inlineStr"/>
-      <c r="D666" t="inlineStr"/>
-      <c r="E666" t="inlineStr"/>
+          <t>Instrumento recolección</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Formulario EBC - PACCP Final</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/spreadsheets/d/1qsclq1ogNVWTc6Sh7swGgV-k7DZr-Wnj/edit?usp=drive_link&amp;ouid=105090632649587320414&amp;rtpof=true&amp;sd=true</t>
+        </is>
+      </c>
     </row>
     <row r="667">
       <c r="A667" t="n">
         <v>118</v>
       </c>
-      <c r="B667" t="inlineStr"/>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Base de datos</t>
+        </is>
+      </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr"/>
       <c r="E667" t="inlineStr"/>
@@ -22500,7 +22520,11 @@
       <c r="A668" t="n">
         <v>118</v>
       </c>
-      <c r="B668" t="inlineStr"/>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Informe cuantitativo</t>
+        </is>
+      </c>
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr"/>
       <c r="E668" t="inlineStr"/>
@@ -22516,32 +22540,16 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>119</v>
-      </c>
-      <c r="B670" t="inlineStr">
-        <is>
-          <t>Carpeta archivos</t>
-        </is>
-      </c>
-      <c r="C670" t="inlineStr">
-        <is>
-          <t>Productos finales Festival de Verano 2025</t>
-        </is>
-      </c>
-      <c r="D670" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/14Ap2CtsPvGqgr55CTIh_z0MO3XnfklKi?usp=sharing</t>
-        </is>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="B670" t="inlineStr"/>
+      <c r="C670" t="inlineStr"/>
+      <c r="D670" t="inlineStr"/>
+      <c r="E670" t="inlineStr"/>
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B671" t="inlineStr"/>
       <c r="C671" t="inlineStr"/>
@@ -22552,10 +22560,26 @@
       <c r="A672" t="n">
         <v>119</v>
       </c>
-      <c r="B672" t="inlineStr"/>
-      <c r="C672" t="inlineStr"/>
-      <c r="D672" t="inlineStr"/>
-      <c r="E672" t="inlineStr"/>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Carpeta archivos</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Productos finales Festival de Verano 2025</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/14Ap2CtsPvGqgr55CTIh_z0MO3XnfklKi?usp=sharing</t>
+        </is>
+      </c>
     </row>
     <row r="673">
       <c r="A673" t="n">
@@ -22586,53 +22610,21 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>120</v>
-      </c>
-      <c r="B676" t="inlineStr">
-        <is>
-          <t>Carpeta archivos</t>
-        </is>
-      </c>
-      <c r="C676" t="inlineStr">
-        <is>
-          <t>Productos finales Concurso Internacional de Violín 2025</t>
-        </is>
-      </c>
-      <c r="D676" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/114QuIa8ZzjC_GNjRUVggtFVTN3y_zOAL?usp=sharing</t>
-        </is>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="B676" t="inlineStr"/>
+      <c r="C676" t="inlineStr"/>
+      <c r="D676" t="inlineStr"/>
+      <c r="E676" t="inlineStr"/>
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>120</v>
-      </c>
-      <c r="B677" t="inlineStr">
-        <is>
-          <t>Carpeta archivos</t>
-        </is>
-      </c>
-      <c r="C677" t="inlineStr">
-        <is>
-          <t>Productos finales Bienal Internacional de Arte y Ciudad BOG25</t>
-        </is>
-      </c>
-      <c r="D677" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/17Bi6a6nKxYmJNqTEWtIH6lYiXMxIECYi?usp=sharing</t>
-        </is>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="B677" t="inlineStr"/>
+      <c r="C677" t="inlineStr"/>
+      <c r="D677" t="inlineStr"/>
+      <c r="E677" t="inlineStr"/>
     </row>
     <row r="678">
       <c r="A678" t="n">
@@ -22645,7 +22637,7 @@
       </c>
       <c r="C678" t="inlineStr">
         <is>
-          <t>Productos finales Navidad es Cultura 2025</t>
+          <t>Productos finales Concurso Internacional de Violín 2025</t>
         </is>
       </c>
       <c r="D678" t="inlineStr">
@@ -22655,7 +22647,7 @@
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rb7lrObK-r5g1iF6SsaYKbR-J_K7nLy-?usp=sharing</t>
+          <t>https://drive.google.com/drive/folders/114QuIa8ZzjC_GNjRUVggtFVTN3y_zOAL?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -22663,19 +22655,51 @@
       <c r="A679" t="n">
         <v>120</v>
       </c>
-      <c r="B679" t="inlineStr"/>
-      <c r="C679" t="inlineStr"/>
-      <c r="D679" t="inlineStr"/>
-      <c r="E679" t="inlineStr"/>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Carpeta archivos</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Productos finales Bienal Internacional de Arte y Ciudad BOG25</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/17Bi6a6nKxYmJNqTEWtIH6lYiXMxIECYi?usp=sharing</t>
+        </is>
+      </c>
     </row>
     <row r="680">
       <c r="A680" t="n">
         <v>120</v>
       </c>
-      <c r="B680" t="inlineStr"/>
-      <c r="C680" t="inlineStr"/>
-      <c r="D680" t="inlineStr"/>
-      <c r="E680" t="inlineStr"/>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Carpeta archivos</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Productos finales Navidad es Cultura 2025</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1rb7lrObK-r5g1iF6SsaYKbR-J_K7nLy-?usp=sharing</t>
+        </is>
+      </c>
     </row>
     <row r="681">
       <c r="A681" t="n">
@@ -22688,53 +22712,21 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>121</v>
-      </c>
-      <c r="B682" t="inlineStr">
-        <is>
-          <t>Visualización</t>
-        </is>
-      </c>
-      <c r="C682" t="inlineStr">
-        <is>
-          <t>Tablero Encuesta</t>
-        </is>
-      </c>
-      <c r="D682" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr">
-        <is>
-          <t>https://lookerstudio.google.com/reporting/ccbecff5-f250-4a21-b1f8-5290632c1187/page/p_shhgwuepsd</t>
-        </is>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="B682" t="inlineStr"/>
+      <c r="C682" t="inlineStr"/>
+      <c r="D682" t="inlineStr"/>
+      <c r="E682" t="inlineStr"/>
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>121</v>
-      </c>
-      <c r="B683" t="inlineStr">
-        <is>
-          <t>Presentación</t>
-        </is>
-      </c>
-      <c r="C683" t="inlineStr">
-        <is>
-          <t>Instrucciones sobre registro de información</t>
-        </is>
-      </c>
-      <c r="D683" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1gbIyrWH8cK07q00yoPBs9D8IWYNv4P2I/view?usp=drive_link</t>
-        </is>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="B683" t="inlineStr"/>
+      <c r="C683" t="inlineStr"/>
+      <c r="D683" t="inlineStr"/>
+      <c r="E683" t="inlineStr"/>
     </row>
     <row r="684">
       <c r="A684" t="n">
@@ -22742,12 +22734,12 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>Prototipo para registro</t>
+          <t>Tablero Encuesta</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
@@ -22757,7 +22749,7 @@
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>https://www.prototipos-sicc.com/app/barrios_vivos/explorar</t>
+          <t>https://lookerstudio.google.com/reporting/ccbecff5-f250-4a21-b1f8-5290632c1187/page/p_shhgwuepsd</t>
         </is>
       </c>
     </row>
@@ -22767,12 +22759,12 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
         <is>
-          <t>Tablero de seguimiento</t>
+          <t>Instrucciones sobre registro de información</t>
         </is>
       </c>
       <c r="D685" t="inlineStr">
@@ -22782,7 +22774,7 @@
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>https://lookerstudio.google.com/reporting/a1e266a6-ed1a-4500-8776-58e82d1d7746/page/p_pjg06p6njd</t>
+          <t>https://drive.google.com/file/d/1gbIyrWH8cK07q00yoPBs9D8IWYNv4P2I/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -22792,12 +22784,12 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Audiovisual</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>Vídeo tutoriales para registro</t>
+          <t>Prototipo para registro</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
@@ -22807,22 +22799,22 @@
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1Cuy0w3cr883zTx_4X1n4TquCUCnheBRm</t>
+          <t>https://www.prototipos-sicc.com/app/barrios_vivos/explorar</t>
         </is>
       </c>
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>Presentación final</t>
+          <t>Tablero de seguimiento</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
@@ -22832,22 +22824,22 @@
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1f6sPy_pAB5aZpB_kvra4Qy4YiKsiGjgR/view?usp=drive_link</t>
+          <t>https://lookerstudio.google.com/reporting/a1e266a6-ed1a-4500-8776-58e82d1d7746/page/p_pjg06p6njd</t>
         </is>
       </c>
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Audiovisual</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>Presentación final</t>
+          <t>Vídeo tutoriales para registro</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
@@ -22857,22 +22849,22 @@
       </c>
       <c r="E688" t="inlineStr">
         <is>
-          <t>https://docs.google.com/presentation/d/1BogTIIMdH15s1-pa4Z9qN-RIW_VTct_g/edit?slide=id.p1#slide=id.p1</t>
+          <t>https://drive.google.com/drive/folders/1Cuy0w3cr883zTx_4X1n4TquCUCnheBRm</t>
         </is>
       </c>
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Anexo</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>Anexo resultados comparativos</t>
+          <t>Presentación final</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
@@ -22882,17 +22874,17 @@
       </c>
       <c r="E689" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/11YGZTE7pzMI4lDBZmvYiq5Xq9TwCE1z4/edit?usp=drive_link&amp;ouid=114299960211627169695&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1f6sPy_pAB5aZpB_kvra4Qy4YiKsiGjgR/view?usp=drive_link</t>
         </is>
       </c>
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>Infografía</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
@@ -22907,30 +22899,34 @@
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1VhroKpPxgqcqQso3fwqBLmJ5zbwmJ8od/view?usp=share_link</t>
+          <t>https://docs.google.com/presentation/d/1BogTIIMdH15s1-pa4Z9qN-RIW_VTct_g/edit?slide=id.p1#slide=id.p1</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Anexo</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>Diseño de experimento económico</t>
+          <t>Anexo resultados comparativos</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/spreadsheets/d/11YGZTE7pzMI4lDBZmvYiq5Xq9TwCE1z4/edit?usp=drive_link&amp;ouid=114299960211627169695&amp;rtpof=true&amp;sd=true</t>
+        </is>
+      </c>
     </row>
     <row r="692">
       <c r="A692" t="n">
@@ -22938,20 +22934,24 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
+          <t>Infografía</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>Cálculo de consumo de agua en ducha por factura</t>
+          <t>Presentación final</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1VhroKpPxgqcqQso3fwqBLmJ5zbwmJ8od/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="693">
       <c r="A693" t="n">
@@ -22959,12 +22959,12 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Otro</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>Datos EAAB por Barrio para experimento</t>
+          <t>Diseño de experimento económico</t>
         </is>
       </c>
       <c r="D693" t="inlineStr">
@@ -22980,12 +22980,12 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Infografía</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>Datos de hitos Barrios Vivos Agua</t>
+          <t>Cálculo de consumo de agua en ducha por factura</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
@@ -23001,12 +23001,12 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>Plan de trabajo</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>Cronograma Investigación Agua</t>
+          <t>Datos EAAB por Barrio para experimento</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
@@ -23018,41 +23018,37 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Infografía</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>Presentación final</t>
+          <t>Datos de hitos Barrios Vivos Agua</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1KnbyFYzDxdGfLHJqZDXjhrrUnvwF8O0D/view?usp=share_link</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Informe cuantitativo</t>
+          <t>Plan de trabajo</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>Tablas de salida</t>
+          <t>Cronograma Investigación Agua</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
@@ -23068,12 +23064,12 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>Carpeta archivos</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>ICC Distritos Creativos 2025</t>
+          <t>Presentación final</t>
         </is>
       </c>
       <c r="D698" t="inlineStr">
@@ -23081,7 +23077,11 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E698" t="inlineStr"/>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1KnbyFYzDxdGfLHJqZDXjhrrUnvwF8O0D/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="699">
       <c r="A699" t="n">
@@ -23089,17 +23089,17 @@
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe cuantitativo</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
         <is>
-          <t>Formulario ICC Distritos Creativos 2025</t>
+          <t>Tablas de salida</t>
         </is>
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -23110,33 +23110,33 @@
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>Plan de trabajo</t>
+          <t>Carpeta archivos</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>Cronograma ICC Distritos Creativos</t>
+          <t>ICC Distritos Creativos 2025</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="E700" t="inlineStr"/>
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>Informe de caracterización con fuentes secundarias</t>
+          <t>Formulario ICC Distritos Creativos 2025</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
@@ -23144,40 +23144,32 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1nqXIcpjznaD1Dn8fjBR_fg7L2XdFwKsg/view?usp=share_link</t>
-        </is>
-      </c>
+      <c r="E701" t="inlineStr"/>
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Plan de trabajo</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tablero de recorrido por espacio púbilco del centro </t>
+          <t>Cronograma ICC Distritos Creativos</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>https://sdcrd.maps.arcgis.com/apps/dashboards/f5ba03060ca94dfa8d4fee25f0de6d7f</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23186,28 +23178,32 @@
       </c>
       <c r="C703" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tablero de recorrido por espacio púbilco del centro </t>
+          <t>Informe de caracterización con fuentes secundarias</t>
         </is>
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1nqXIcpjznaD1Dn8fjBR_fg7L2XdFwKsg/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t xml:space="preserve">Tablero de recorrido por espacio púbilco del centro </t>
         </is>
       </c>
       <c r="D704" t="inlineStr">
@@ -23217,34 +23213,30 @@
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1NsVGUlWsADXoKnEO31ub8Cp0Krp9Aig3/view?usp=drive_link</t>
+          <t>https://sdcrd.maps.arcgis.com/apps/dashboards/f5ba03060ca94dfa8d4fee25f0de6d7f</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>Anexo</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>Anexo de definición</t>
+          <t xml:space="preserve">Tablero de recorrido por espacio púbilco del centro </t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1yZIHrgUGq2Lu0TFlzzyGvCS7RXjuxd1M/view?usp=drive_link</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
     </row>
     <row r="706">
       <c r="A706" t="n">
@@ -23252,12 +23244,12 @@
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>Formulario sondeo</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
@@ -23267,7 +23259,7 @@
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1AVJBnJQld7Uyna3WW04TEPkFOQQqFlQl/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1NsVGUlWsADXoKnEO31ub8Cp0Krp9Aig3/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -23275,19 +23267,51 @@
       <c r="A707" t="n">
         <v>128</v>
       </c>
-      <c r="B707" t="inlineStr"/>
-      <c r="C707" t="inlineStr"/>
-      <c r="D707" t="inlineStr"/>
-      <c r="E707" t="inlineStr"/>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Anexo</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Anexo de definición</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1yZIHrgUGq2Lu0TFlzzyGvCS7RXjuxd1M/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="708">
       <c r="A708" t="n">
         <v>128</v>
       </c>
-      <c r="B708" t="inlineStr"/>
-      <c r="C708" t="inlineStr"/>
-      <c r="D708" t="inlineStr"/>
-      <c r="E708" t="inlineStr"/>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Instrumento recolección</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Formulario sondeo</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1AVJBnJQld7Uyna3WW04TEPkFOQQqFlQl/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" t="n">
@@ -23300,62 +23324,34 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>129</v>
-      </c>
-      <c r="B710" t="inlineStr">
-        <is>
-          <t>Informe final</t>
-        </is>
-      </c>
-      <c r="C710" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Análisis de impacto de la implementación de los Laboratorios de Bienestar a adolescentes: Comparación de encuestas pre y post de la implementación del laboratorio: “El Viaje Hacia Dentro de Mi” - Estrategia EstarBien Bogotá </t>
-        </is>
-      </c>
-      <c r="D710" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1R8tXuWA5XQrs_U1P2LAakV8WjHZp-Hyc/view?usp=share_link</t>
-        </is>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="B710" t="inlineStr"/>
+      <c r="C710" t="inlineStr"/>
+      <c r="D710" t="inlineStr"/>
+      <c r="E710" t="inlineStr"/>
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>129</v>
-      </c>
-      <c r="B711" t="inlineStr">
-        <is>
-          <t>Plan de trabajo</t>
-        </is>
-      </c>
-      <c r="C711" t="inlineStr">
-        <is>
-          <t>Plan de investigación</t>
-        </is>
-      </c>
-      <c r="D711" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="B711" t="inlineStr"/>
+      <c r="C711" t="inlineStr"/>
+      <c r="D711" t="inlineStr"/>
       <c r="E711" t="inlineStr"/>
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>Matriz de preguntas de la EBC</t>
+          <t xml:space="preserve">Análisis de impacto de la implementación de los Laboratorios de Bienestar a adolescentes: Comparación de encuestas pre y post de la implementación del laboratorio: “El Viaje Hacia Dentro de Mi” - Estrategia EstarBien Bogotá </t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
@@ -23365,38 +23361,34 @@
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+          <t>https://drive.google.com/file/d/1R8tXuWA5XQrs_U1P2LAakV8WjHZp-Hyc/view?usp=share_link</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Plan de trabajo</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>Presentación final</t>
+          <t>Plan de investigación</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1Ez5bU0fGKborxl5_zyUc27muZZizMtFC/view?usp=share_link</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -23405,28 +23397,32 @@
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>Encuesta de recolección de fuentes primarias</t>
+          <t>Matriz de preguntas de la EBC</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Cultura Metro - Estado del Arte</t>
+          <t>Presentación final</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -23436,52 +23432,80 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>https://docs.google.com/document/d/1TvqbXkunNvyWYuMDu2TZ_rwJeAI2fjFR/edit?usp=sharing&amp;ouid=100772003525119686921&amp;rtpof=true&amp;sd=true</t>
+          <t>https://drive.google.com/file/d/1Ez5bU0fGKborxl5_zyUc27muZZizMtFC/view?usp=share_link</t>
         </is>
       </c>
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presentación Final </t>
+          <t>Encuesta de recolección de fuentes primarias</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/16AYD-Y9HF8O45rYDxH6a_pgEbUjv_Ofo/view?usp=drive_link</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>134</v>
-      </c>
-      <c r="B717" t="inlineStr"/>
-      <c r="C717" t="inlineStr"/>
-      <c r="D717" t="inlineStr"/>
-      <c r="E717" t="inlineStr"/>
+        <v>132</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Informe final</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Cultura Metro - Estado del Arte</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/document/d/1TvqbXkunNvyWYuMDu2TZ_rwJeAI2fjFR/edit?usp=sharing&amp;ouid=100772003525119686921&amp;rtpof=true&amp;sd=true</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>134</v>
-      </c>
-      <c r="B718" t="inlineStr"/>
-      <c r="C718" t="inlineStr"/>
-      <c r="D718" t="inlineStr"/>
-      <c r="E718" t="inlineStr"/>
+        <v>133</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Presentación</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentación Final </t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/16AYD-Y9HF8O45rYDxH6a_pgEbUjv_Ofo/view?usp=drive_link</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" t="n">
@@ -23514,80 +23538,48 @@
       <c r="A722" t="n">
         <v>134</v>
       </c>
-      <c r="B722" t="inlineStr">
-        <is>
-          <t>Visualización</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr">
-        <is>
-          <t>Tablero invitados ECCI 2025 - Seguimiento</t>
-        </is>
-      </c>
-      <c r="D722" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr">
-        <is>
-          <t>https://lookerstudio.google.com/reporting/49195a24-bd9a-4773-af8a-966bb697f78b/page/p_pjg06p6njd</t>
-        </is>
-      </c>
+      <c r="B722" t="inlineStr"/>
+      <c r="C722" t="inlineStr"/>
+      <c r="D722" t="inlineStr"/>
+      <c r="E722" t="inlineStr"/>
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>135</v>
-      </c>
-      <c r="B723" t="inlineStr">
-        <is>
-          <t>Informe final</t>
-        </is>
-      </c>
-      <c r="C723" t="inlineStr">
-        <is>
-          <t>Marco conceptual</t>
-        </is>
-      </c>
-      <c r="D723" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/12I-YN44-_0suC2dpHX3vOLYgHwHTHA-E/view?usp=share_link</t>
-        </is>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="B723" t="inlineStr"/>
+      <c r="C723" t="inlineStr"/>
+      <c r="D723" t="inlineStr"/>
+      <c r="E723" t="inlineStr"/>
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t xml:space="preserve">índice de reconciliación y paz </t>
+          <t>Tablero invitados ECCI 2025 - Seguimiento</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ySdEC1LyX43LPMZdqi2vBiSWXoQRieJH/view?usp=share_link</t>
+          <t>https://lookerstudio.google.com/reporting/49195a24-bd9a-4773-af8a-966bb697f78b/page/p_pjg06p6njd</t>
         </is>
       </c>
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
@@ -23596,30 +23588,32 @@
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento Desarrollo Técnico Normativo y misional del enfoque de Cultura Ciudadana para la movilidad
-</t>
+          <t>Marco conceptual</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12I-YN44-_0suC2dpHX3vOLYgHwHTHA-E/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Informe final</t>
+          <t>Instrumento recolección</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estado del arte y de la práctica sobre problemáticas relacionadas a cultura ciudadana y movilidad 
-</t>
+          <t xml:space="preserve">índice de reconciliación y paz </t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
@@ -23629,7 +23623,7 @@
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1l3CBDIXbCVbiG153wP35kkD4Q44DZbI1/view?usp=share_link</t>
+          <t>https://drive.google.com/file/d/1ySdEC1LyX43LPMZdqi2vBiSWXoQRieJH/view?usp=share_link</t>
         </is>
       </c>
     </row>
@@ -23639,12 +23633,13 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Mapa/Geovisor</t>
+          <t>Informe final</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>Geovisor Movilidad</t>
+          <t xml:space="preserve">Documento Desarrollo Técnico Normativo y misional del enfoque de Cultura Ciudadana para la movilidad
+</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
@@ -23652,15 +23647,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E727" t="inlineStr">
-        <is>
-          <t>https://www.arcgis.com/apps/dashboards/3a8a858de18047528174d7bc158b4b42</t>
-        </is>
-      </c>
+      <c r="E727" t="inlineStr"/>
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
@@ -23669,7 +23660,8 @@
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>Informe final de mediciones</t>
+          <t xml:space="preserve">Estado del arte y de la práctica sobre problemáticas relacionadas a cultura ciudadana y movilidad 
+</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
@@ -23679,32 +23671,32 @@
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1liHn1t_9w1D5ry0UIfT6kxLszVuyErB_/view?usp=drive_link</t>
+          <t>https://drive.google.com/file/d/1l3CBDIXbCVbiG153wP35kkD4Q44DZbI1/view?usp=share_link</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Mapa/Geovisor</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>Tablero de resultados</t>
+          <t>Geovisor Movilidad</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/view?r=eyJrIjoiOWYwOThhMjMtOTBjZC00ZGY5LThhYjktMTY5OWYzYWI0ZDJjIiwidCI6IjRmNzkzOWM3LWFhNjAtNDliZC05YjdiLTZmODFjMzdkMWIzNyJ9&amp;pageName=ef377ed828063259b15e</t>
+          <t>https://www.arcgis.com/apps/dashboards/3a8a858de18047528174d7bc158b4b42</t>
         </is>
       </c>
     </row>
@@ -23714,20 +23706,70 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
+          <t>Informe final</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Informe final de mediciones</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1liHn1t_9w1D5ry0UIfT6kxLszVuyErB_/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="n">
+        <v>137</v>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Visualización</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Tablero de resultados</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/view?r=eyJrIjoiOWYwOThhMjMtOTBjZC00ZGY5LThhYjktMTY5OWYzYWI0ZDJjIiwidCI6IjRmNzkzOWM3LWFhNjAtNDliZC05YjdiLTZmODFjMzdkMWIzNyJ9&amp;pageName=ef377ed828063259b15e</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="n">
+        <v>137</v>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
           <t>Base de datos</t>
         </is>
       </c>
-      <c r="C730" t="inlineStr">
+      <c r="C732" t="inlineStr">
         <is>
           <t>Datos de encuestas</t>
         </is>
       </c>
-      <c r="D730" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr">
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/1rX2RfuDon4SukoBpHxRg7m9fnL6_1Jw2/edit?usp=drive_link&amp;ouid=114299960211627169695&amp;rtpof=true&amp;sd=true</t>
         </is>

</xml_diff>

<commit_message>
Update investigaciones, i130 v2
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -3309,7 +3309,7 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -26044,12 +26044,12 @@
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>Matriz de preguntas de la EBC</t>
+          <t>Presentación resumen de resultados</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -26059,7 +26059,7 @@
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+          <t>https://docs.google.com/presentation/d/1bPLTlrkQNn8G8vEepHLs5l3QTNfF8usV/edit?slide=id.p1#slide=id.p1</t>
         </is>
       </c>
     </row>
@@ -26067,10 +26067,26 @@
       <c r="A717" t="n">
         <v>130</v>
       </c>
-      <c r="B717" t="inlineStr"/>
-      <c r="C717" t="inlineStr"/>
-      <c r="D717" t="inlineStr"/>
-      <c r="E717" t="inlineStr"/>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Instrumento recolección</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Matriz de preguntas de la EBC</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" t="n">

</xml_diff>

<commit_message>
Update investigaciones, i130 v3, nueva ppt
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -3309,7 +3309,7 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -26059,7 +26059,7 @@
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>https://docs.google.com/presentation/d/1bPLTlrkQNn8G8vEepHLs5l3QTNfF8usV/edit?slide=id.p1#slide=id.p1</t>
+          <t>https://docs.google.com/presentation/d/1eq2OlrJJGnYvh_AV6hq9vvACrpBeUkTo/edit?slide=id.p1#slide=id.p1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update investigaciones, i130 v4, db respuestas
</commit_message>
<xml_diff>
--- a/content/data/investigaciones/investigaciones.xlsx
+++ b/content/data/investigaciones/investigaciones.xlsx
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="O35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -3309,7 +3309,7 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -26019,12 +26019,12 @@
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Visualización</t>
+          <t>Presentación</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>Tabero de Resultados</t>
+          <t>Presentación resumen de resultados</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>https://observatoriocultura.github.io/observatorio/#/ebc/encuesta-cultura-ciudadana-2025</t>
+          <t>https://docs.google.com/presentation/d/1eq2OlrJJGnYvh_AV6hq9vvACrpBeUkTo/edit?slide=id.p1#slide=id.p1</t>
         </is>
       </c>
     </row>
@@ -26044,12 +26044,12 @@
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Presentación</t>
+          <t>Visualización</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>Presentación resumen de resultados</t>
+          <t>Tabero de Resultados</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -26059,7 +26059,7 @@
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>https://docs.google.com/presentation/d/1eq2OlrJJGnYvh_AV6hq9vvACrpBeUkTo/edit?slide=id.p1#slide=id.p1</t>
+          <t>https://observatoriocultura.github.io/observatorio/#/ebc/encuesta-cultura-ciudadana-2025</t>
         </is>
       </c>
     </row>
@@ -26069,12 +26069,12 @@
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>Instrumento recolección</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>Matriz de preguntas de la EBC</t>
+          <t>Datos detallados de respuestas</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
@@ -26084,7 +26084,7 @@
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+          <t>https://docs.google.com/spreadsheets/d/1nCsuCpG7YJ-PQ7ilHtNdGahIDfNHcHDT/edit?usp=drive_link&amp;ouid=114299960211627169695&amp;rtpof=true&amp;sd=true</t>
         </is>
       </c>
     </row>
@@ -26092,10 +26092,26 @@
       <c r="A718" t="n">
         <v>130</v>
       </c>
-      <c r="B718" t="inlineStr"/>
-      <c r="C718" t="inlineStr"/>
-      <c r="D718" t="inlineStr"/>
-      <c r="E718" t="inlineStr"/>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Instrumento recolección</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Matriz de preguntas de la EBC</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1DBDvo9ZxCKI-N5iG-XNns-ILD2S1UEMe/view?usp=share_link</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" t="n">

</xml_diff>